<commit_message>
atividae grafico de calor
</commit_message>
<xml_diff>
--- a/1Semestre/GerenciamentoDeProjetos/Desempenho da Equipe de Desenvolvimento.xlsx
+++ b/1Semestre/GerenciamentoDeProjetos/Desempenho da Equipe de Desenvolvimento.xlsx
@@ -615,8 +615,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B7">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF57BB8A"/>
+        <color rgb="FFFFD666"/>
+        <color rgb="FFE67C73"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B2:D7">
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>